<commit_message>
Fix results folder structure: correct naming and no nesting
</commit_message>
<xml_diff>
--- a/get_results/results/aim.pat003.v1.20260422.thighs_dixon3pt_t2slice/results.xlsx
+++ b/get_results/results/aim.pat003.v1.20260422.thighs_dixon3pt_t2slice/results.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -509,7 +509,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -542,7 +542,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -575,7 +575,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -641,7 +641,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -674,7 +674,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -707,7 +707,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -740,7 +740,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -773,7 +773,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -806,7 +806,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -839,7 +839,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -872,7 +872,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -905,7 +905,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -938,7 +938,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -971,7 +971,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1613,7 +1613,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1675,7 +1675,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2450,7 +2450,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2574,7 +2574,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2853,7 +2853,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2946,7 +2946,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -3070,7 +3070,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -3101,7 +3101,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -3163,7 +3163,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -3349,7 +3349,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -3442,7 +3442,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -3473,7 +3473,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -3504,7 +3504,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -3628,7 +3628,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3659,7 +3659,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -3690,7 +3690,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -3752,7 +3752,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3845,7 +3845,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3876,7 +3876,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3907,7 +3907,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3938,7 +3938,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3969,7 +3969,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -4000,7 +4000,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -4124,7 +4124,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -4155,7 +4155,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -4186,7 +4186,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -4217,7 +4217,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -4248,7 +4248,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -4279,7 +4279,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -4372,7 +4372,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -4465,7 +4465,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -4527,7 +4527,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -4589,7 +4589,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -4620,7 +4620,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -4682,7 +4682,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -4713,7 +4713,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4744,7 +4744,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -4775,7 +4775,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4837,7 +4837,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -4868,7 +4868,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -4899,7 +4899,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -4930,7 +4930,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -4961,7 +4961,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4992,7 +4992,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -5054,7 +5054,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -5085,7 +5085,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -5116,7 +5116,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -5147,7 +5147,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -5178,7 +5178,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -5271,7 +5271,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -5302,7 +5302,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -5426,7 +5426,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -5457,7 +5457,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -5488,7 +5488,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -5519,7 +5519,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -5550,7 +5550,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -5581,7 +5581,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -5612,7 +5612,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -5643,7 +5643,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -5674,7 +5674,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -5705,7 +5705,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -5736,7 +5736,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -5767,7 +5767,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -5798,7 +5798,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -5829,7 +5829,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -5860,7 +5860,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -5891,7 +5891,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -5922,7 +5922,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -5953,7 +5953,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -5984,7 +5984,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -6015,7 +6015,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -6077,7 +6077,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -6108,7 +6108,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -6139,7 +6139,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -6232,7 +6232,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -6294,7 +6294,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -6325,7 +6325,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -6356,7 +6356,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -6387,7 +6387,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -6418,7 +6418,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -6449,7 +6449,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -6511,7 +6511,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -6542,7 +6542,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -6573,7 +6573,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -6604,7 +6604,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -6635,7 +6635,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -6697,7 +6697,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -6728,7 +6728,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -6759,7 +6759,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -6821,7 +6821,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -6852,7 +6852,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -6883,7 +6883,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D207" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D208" t="n">
@@ -6945,7 +6945,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -6976,7 +6976,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -7038,7 +7038,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -7069,7 +7069,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -7162,7 +7162,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D216" t="n">
@@ -7193,7 +7193,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D217" t="n">
@@ -7224,7 +7224,7 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D218" t="n">
@@ -7255,7 +7255,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D219" t="n">
@@ -7286,7 +7286,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D220" t="n">
@@ -7317,7 +7317,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D221" t="n">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D222" t="n">
@@ -7379,7 +7379,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D223" t="n">
@@ -7410,7 +7410,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -7441,7 +7441,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D225" t="n">
@@ -7472,7 +7472,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -7503,7 +7503,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -7534,7 +7534,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D228" t="n">
@@ -7565,7 +7565,7 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D229" t="n">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D230" t="n">
@@ -7627,7 +7627,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D231" t="n">
@@ -7658,7 +7658,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D232" t="n">
@@ -7689,7 +7689,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D233" t="n">
@@ -7720,7 +7720,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D234" t="n">
@@ -7751,7 +7751,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D235" t="n">
@@ -7782,7 +7782,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D236" t="n">
@@ -7813,7 +7813,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D238" t="n">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -7906,7 +7906,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -7937,7 +7937,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -7968,7 +7968,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -7999,7 +7999,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -8030,7 +8030,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -8061,7 +8061,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -8092,7 +8092,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -8123,7 +8123,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -8154,7 +8154,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -8185,7 +8185,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D249" t="n">
@@ -8216,7 +8216,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -8247,7 +8247,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -8278,7 +8278,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -8309,7 +8309,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D253" t="n">
@@ -8340,7 +8340,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D254" t="n">
@@ -8371,7 +8371,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -8402,7 +8402,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D256" t="n">
@@ -8433,7 +8433,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D257" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D258" t="n">
@@ -8495,7 +8495,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -8526,7 +8526,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -8557,7 +8557,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D261" t="n">
@@ -8588,7 +8588,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D262" t="n">
@@ -8625,7 +8625,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -8662,7 +8662,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -8699,7 +8699,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -8730,7 +8730,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D266" t="n">
@@ -8767,7 +8767,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D267" t="n">
@@ -8804,7 +8804,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D268" t="n">
@@ -8841,7 +8841,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -8872,7 +8872,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -8909,7 +8909,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -8946,7 +8946,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D272" t="n">
@@ -8977,7 +8977,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -9008,7 +9008,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -9039,7 +9039,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D275" t="n">
@@ -9070,7 +9070,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D276" t="n">
@@ -9107,7 +9107,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D277" t="n">
@@ -9144,7 +9144,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D278" t="n">
@@ -9175,7 +9175,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D279" t="n">
@@ -9212,7 +9212,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -9280,7 +9280,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D282" t="n">
@@ -9311,7 +9311,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D283" t="n">
@@ -9342,7 +9342,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D284" t="n">
@@ -9379,7 +9379,7 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D285" t="n">
@@ -9410,7 +9410,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D286" t="n">
@@ -9441,7 +9441,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D287" t="n">
@@ -9472,7 +9472,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D288" t="n">
@@ -9509,7 +9509,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D289" t="n">
@@ -9546,7 +9546,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -9583,7 +9583,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D292" t="n">
@@ -9651,7 +9651,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D293" t="n">
@@ -9688,7 +9688,7 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D294" t="n">
@@ -9725,7 +9725,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D295" t="n">
@@ -9756,7 +9756,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D296" t="n">
@@ -9793,7 +9793,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D297" t="n">
@@ -9830,7 +9830,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -9861,7 +9861,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D299" t="n">
@@ -9892,7 +9892,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D300" t="n">
@@ -9923,7 +9923,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D301" t="n">
@@ -9960,7 +9960,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D302" t="n">
@@ -9997,7 +9997,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D303" t="n">
@@ -10034,7 +10034,7 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D304" t="n">
@@ -10065,7 +10065,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D305" t="n">
@@ -10102,7 +10102,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D306" t="n">
@@ -10139,7 +10139,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -10176,7 +10176,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D308" t="n">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -10238,7 +10238,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -10275,7 +10275,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D311" t="n">
@@ -10306,7 +10306,7 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D312" t="n">
@@ -10337,7 +10337,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D313" t="n">
@@ -10368,7 +10368,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D314" t="n">
@@ -10405,7 +10405,7 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D315" t="n">
@@ -10442,7 +10442,7 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D316" t="n">
@@ -10479,7 +10479,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D317" t="n">
@@ -10516,7 +10516,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D318" t="n">
@@ -10553,7 +10553,7 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D319" t="n">
@@ -10590,7 +10590,7 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D320" t="n">
@@ -10627,7 +10627,7 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D321" t="n">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D322" t="n">
@@ -10701,7 +10701,7 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D323" t="n">
@@ -10738,7 +10738,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D324" t="n">
@@ -10775,7 +10775,7 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D325" t="n">
@@ -10806,7 +10806,7 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D326" t="n">
@@ -10837,7 +10837,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D327" t="n">
@@ -10874,7 +10874,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D328" t="n">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -10948,7 +10948,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D330" t="n">
@@ -10985,7 +10985,7 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D331" t="n">
@@ -11022,7 +11022,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D332" t="n">
@@ -11059,7 +11059,7 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D333" t="n">
@@ -11096,7 +11096,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D334" t="n">
@@ -11127,7 +11127,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -11164,7 +11164,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D336" t="n">
@@ -11201,7 +11201,7 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D337" t="n">
@@ -11238,7 +11238,7 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D338" t="n">
@@ -11269,7 +11269,7 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D339" t="n">
@@ -11300,7 +11300,7 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D340" t="n">
@@ -11337,7 +11337,7 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D341" t="n">
@@ -11374,7 +11374,7 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D342" t="n">
@@ -11411,7 +11411,7 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D343" t="n">
@@ -11448,7 +11448,7 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D344" t="n">
@@ -11485,7 +11485,7 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D345" t="n">
@@ -11522,7 +11522,7 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D346" t="n">
@@ -11559,7 +11559,7 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D347" t="n">
@@ -11596,7 +11596,7 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D348" t="n">
@@ -11633,7 +11633,7 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D349" t="n">
@@ -11670,7 +11670,7 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D350" t="n">
@@ -11707,7 +11707,7 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D351" t="n">
@@ -11738,7 +11738,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D352" t="n">
@@ -11769,7 +11769,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D353" t="n">
@@ -11806,7 +11806,7 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D354" t="n">
@@ -11843,7 +11843,7 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D355" t="n">
@@ -11880,7 +11880,7 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D356" t="n">
@@ -11917,7 +11917,7 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D357" t="n">
@@ -11954,7 +11954,7 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D358" t="n">
@@ -11991,7 +11991,7 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D359" t="n">
@@ -12028,7 +12028,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D360" t="n">
@@ -12065,7 +12065,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D362" t="n">
@@ -12139,7 +12139,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D363" t="n">
@@ -12176,7 +12176,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D364" t="n">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D365" t="n">
@@ -12238,7 +12238,7 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D366" t="n">
@@ -12275,7 +12275,7 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D367" t="n">
@@ -12312,7 +12312,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D368" t="n">
@@ -12349,7 +12349,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D369" t="n">
@@ -12386,7 +12386,7 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D370" t="n">
@@ -12423,7 +12423,7 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D371" t="n">
@@ -12460,7 +12460,7 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D372" t="n">
@@ -12497,7 +12497,7 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D373" t="n">
@@ -12534,7 +12534,7 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D374" t="n">
@@ -12571,7 +12571,7 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D375" t="n">
@@ -12608,7 +12608,7 @@
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D376" t="n">
@@ -12645,7 +12645,7 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D377" t="n">
@@ -12682,7 +12682,7 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D378" t="n">
@@ -12713,7 +12713,7 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D379" t="n">
@@ -12750,7 +12750,7 @@
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D380" t="n">
@@ -12787,7 +12787,7 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D381" t="n">
@@ -12824,7 +12824,7 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D382" t="n">
@@ -12861,7 +12861,7 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D383" t="n">
@@ -12898,7 +12898,7 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D384" t="n">
@@ -12935,7 +12935,7 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D385" t="n">
@@ -12972,7 +12972,7 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D386" t="n">
@@ -13009,7 +13009,7 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D387" t="n">
@@ -13046,7 +13046,7 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D388" t="n">
@@ -13083,7 +13083,7 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D389" t="n">
@@ -13120,7 +13120,7 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D390" t="n">
@@ -13157,7 +13157,7 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D391" t="n">
@@ -13188,7 +13188,7 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D392" t="n">
@@ -13225,7 +13225,7 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D393" t="n">
@@ -13262,7 +13262,7 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D394" t="n">
@@ -13299,7 +13299,7 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D395" t="n">
@@ -13336,7 +13336,7 @@
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D396" t="n">
@@ -13373,7 +13373,7 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D397" t="n">
@@ -13410,7 +13410,7 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D398" t="n">
@@ -13447,7 +13447,7 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D399" t="n">
@@ -13484,7 +13484,7 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D400" t="n">
@@ -13521,7 +13521,7 @@
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D401" t="n">
@@ -13558,7 +13558,7 @@
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D402" t="n">
@@ -13595,7 +13595,7 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D403" t="n">
@@ -13632,7 +13632,7 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D404" t="n">
@@ -13663,7 +13663,7 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D405" t="n">
@@ -13700,7 +13700,7 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D406" t="n">
@@ -13737,7 +13737,7 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D407" t="n">
@@ -13774,7 +13774,7 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D408" t="n">
@@ -13811,7 +13811,7 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D409" t="n">
@@ -13848,7 +13848,7 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D410" t="n">
@@ -13885,7 +13885,7 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D411" t="n">
@@ -13922,7 +13922,7 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D412" t="n">
@@ -13959,7 +13959,7 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D413" t="n">
@@ -13996,7 +13996,7 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D414" t="n">
@@ -14033,7 +14033,7 @@
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D415" t="n">
@@ -14070,7 +14070,7 @@
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D416" t="n">
@@ -14107,7 +14107,7 @@
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D417" t="n">
@@ -14138,7 +14138,7 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D418" t="n">
@@ -14175,7 +14175,7 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D419" t="n">
@@ -14212,7 +14212,7 @@
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D420" t="n">
@@ -14249,7 +14249,7 @@
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D421" t="n">
@@ -14286,7 +14286,7 @@
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D422" t="n">
@@ -14323,7 +14323,7 @@
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D423" t="n">
@@ -14360,7 +14360,7 @@
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D424" t="n">
@@ -14397,7 +14397,7 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D425" t="n">
@@ -14434,7 +14434,7 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D426" t="n">
@@ -14471,7 +14471,7 @@
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D427" t="n">
@@ -14508,7 +14508,7 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D428" t="n">
@@ -14545,7 +14545,7 @@
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D429" t="n">
@@ -14582,7 +14582,7 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D430" t="n">
@@ -14613,7 +14613,7 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D431" t="n">
@@ -14650,7 +14650,7 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D432" t="n">
@@ -14687,7 +14687,7 @@
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D433" t="n">
@@ -14724,7 +14724,7 @@
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D434" t="n">
@@ -14761,7 +14761,7 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D435" t="n">
@@ -14798,7 +14798,7 @@
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D436" t="n">
@@ -14835,7 +14835,7 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D437" t="n">
@@ -14872,7 +14872,7 @@
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D438" t="n">
@@ -14909,7 +14909,7 @@
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D439" t="n">
@@ -14946,7 +14946,7 @@
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D440" t="n">
@@ -14983,7 +14983,7 @@
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D441" t="n">
@@ -15020,7 +15020,7 @@
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D442" t="n">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D443" t="n">
@@ -15088,7 +15088,7 @@
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D444" t="n">
@@ -15125,7 +15125,7 @@
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D445" t="n">
@@ -15162,7 +15162,7 @@
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D446" t="n">
@@ -15199,7 +15199,7 @@
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D447" t="n">
@@ -15236,7 +15236,7 @@
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D448" t="n">
@@ -15273,7 +15273,7 @@
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D449" t="n">
@@ -15310,7 +15310,7 @@
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D450" t="n">
@@ -15347,7 +15347,7 @@
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D451" t="n">
@@ -15384,7 +15384,7 @@
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D452" t="n">
@@ -15421,7 +15421,7 @@
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D453" t="n">
@@ -15452,7 +15452,7 @@
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D454" t="n">
@@ -15489,7 +15489,7 @@
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D455" t="n">
@@ -15526,7 +15526,7 @@
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D456" t="n">
@@ -15563,7 +15563,7 @@
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D457" t="n">
@@ -15600,7 +15600,7 @@
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D458" t="n">
@@ -15637,7 +15637,7 @@
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D459" t="n">
@@ -15674,7 +15674,7 @@
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D460" t="n">
@@ -15711,7 +15711,7 @@
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D461" t="n">
@@ -15748,7 +15748,7 @@
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D462" t="n">
@@ -15785,7 +15785,7 @@
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D463" t="n">
@@ -15822,7 +15822,7 @@
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D464" t="n">
@@ -15859,7 +15859,7 @@
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D465" t="n">
@@ -15896,7 +15896,7 @@
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D466" t="n">
@@ -15927,7 +15927,7 @@
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D467" t="n">
@@ -15964,7 +15964,7 @@
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D468" t="n">
@@ -16001,7 +16001,7 @@
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D469" t="n">
@@ -16038,7 +16038,7 @@
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>VL_R</t>
         </is>
       </c>
       <c r="D470" t="n">
@@ -16075,7 +16075,7 @@
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>VI_R</t>
         </is>
       </c>
       <c r="D471" t="n">
@@ -16112,7 +16112,7 @@
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>VM_R</t>
         </is>
       </c>
       <c r="D472" t="n">
@@ -16149,7 +16149,7 @@
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>RF_R</t>
         </is>
       </c>
       <c r="D473" t="n">
@@ -16186,7 +16186,7 @@
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>SAR_R</t>
         </is>
       </c>
       <c r="D474" t="n">
@@ -16223,7 +16223,7 @@
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>GRA_R</t>
         </is>
       </c>
       <c r="D475" t="n">
@@ -16260,7 +16260,7 @@
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>SM_R</t>
         </is>
       </c>
       <c r="D476" t="n">
@@ -16291,7 +16291,7 @@
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>ST_R</t>
         </is>
       </c>
       <c r="D477" t="n">
@@ -16328,7 +16328,7 @@
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>BF_R</t>
         </is>
       </c>
       <c r="D478" t="n">
@@ -16365,7 +16365,7 @@
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>BF_SH_R</t>
         </is>
       </c>
       <c r="D479" t="n">
@@ -16396,7 +16396,7 @@
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>AM_R</t>
         </is>
       </c>
       <c r="D480" t="n">
@@ -16433,7 +16433,7 @@
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>AL_R</t>
         </is>
       </c>
       <c r="D481" t="n">
@@ -16470,7 +16470,7 @@
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>AB_R</t>
         </is>
       </c>
       <c r="D482" t="n">
@@ -16507,7 +16507,7 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>VL_L</t>
         </is>
       </c>
       <c r="D483" t="n">
@@ -16544,7 +16544,7 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>VI_L</t>
         </is>
       </c>
       <c r="D484" t="n">
@@ -16581,7 +16581,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>VM_L</t>
         </is>
       </c>
       <c r="D485" t="n">
@@ -16618,7 +16618,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>LABEL_17</t>
+          <t>RF_L</t>
         </is>
       </c>
       <c r="D486" t="n">
@@ -16655,7 +16655,7 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>LABEL_18</t>
+          <t>SAR_L</t>
         </is>
       </c>
       <c r="D487" t="n">
@@ -16692,7 +16692,7 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>LABEL_19</t>
+          <t>GRA_L</t>
         </is>
       </c>
       <c r="D488" t="n">
@@ -16729,7 +16729,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>LABEL_20</t>
+          <t>SM_L</t>
         </is>
       </c>
       <c r="D489" t="n">
@@ -16760,7 +16760,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>LABEL_21</t>
+          <t>ST_L</t>
         </is>
       </c>
       <c r="D490" t="n">
@@ -16797,7 +16797,7 @@
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>LABEL_22</t>
+          <t>BF_L</t>
         </is>
       </c>
       <c r="D491" t="n">
@@ -16834,7 +16834,7 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>LABEL_23</t>
+          <t>BF_SH_L</t>
         </is>
       </c>
       <c r="D492" t="n">
@@ -16865,7 +16865,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>LABEL_24</t>
+          <t>AM_L</t>
         </is>
       </c>
       <c r="D493" t="n">
@@ -16902,7 +16902,7 @@
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>LABEL_25</t>
+          <t>AL_L</t>
         </is>
       </c>
       <c r="D494" t="n">
@@ -16939,7 +16939,7 @@
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>LABEL_26</t>
+          <t>AB_L</t>
         </is>
       </c>
       <c r="D495" t="n">

</xml_diff>